<commit_message>
feat(engine): improve natural example translation drafts
'이 예문에서 ...' 형태의 약한 fallback 감소
achieve / provide / prevent / improve / reduce / maintain 등 동사 패턴 추가
noun_phrases.json 추가
verb_patterns.json 추가
</commit_message>
<xml_diff>
--- a/data/words_v3_exampleko_502_1001.xlsx
+++ b/data/words_v3_exampleko_502_1001.xlsx
@@ -483,7 +483,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H3000"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.39999961853027" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.39999961853027"/>
   <cols>
     <col width="18" customWidth="1" style="29" min="1" max="1"/>
     <col width="24" customWidth="1" style="29" min="2" max="2"/>
@@ -37555,7 +37555,7 @@
       </c>
       <c r="D1002" t="inlineStr">
         <is>
-          <t>일부 textile fabrics은 내용이나 실질이 부족합니다.  [초안]</t>
+          <t>일부 직물은 내용이나 실질이 부족합니다.  [초안]</t>
         </is>
       </c>
       <c r="E1002" t="inlineStr">
@@ -37593,7 +37593,7 @@
       </c>
       <c r="D1003" t="inlineStr">
         <is>
-          <t>일부 주민들은 그 제안이 사실보다 감정에 치우쳐 있다며 이의를 제기했습니다.  [초안]</t>
+          <t>일부 주민들은 그 제안이 사실보다 감정에 치우쳐 있다며 이의를 제기했습니다.</t>
         </is>
       </c>
       <c r="E1003" t="inlineStr">
@@ -37631,7 +37631,7 @@
       </c>
       <c r="D1004" t="inlineStr">
         <is>
-          <t>어떤 사람들은 자신이 사는 도시 안에서만 유명합니다.  [초안]</t>
+          <t>어떤 사람들은 자신이 사는 도시 안에서만 유명합니다.</t>
         </is>
       </c>
       <c r="E1004" t="inlineStr">
@@ -37669,7 +37669,7 @@
       </c>
       <c r="D1005" t="inlineStr">
         <is>
-          <t>어떤 사람들은 sports.에 지나치게 몰두합니다.  [초안]</t>
+          <t>어떤 사람들은 스포츠에 지나치게 몰두합니다.</t>
         </is>
       </c>
       <c r="E1005" t="inlineStr">
@@ -37823,7 +37823,7 @@
       </c>
       <c r="D1009" t="inlineStr">
         <is>
-          <t>사회적 긴장이 최근의 정치적인 위기로 인해 고조되었습니다.</t>
+          <t>최근의 정치적인 위기로 인해 사회적 긴장이 고조되었습니다.</t>
         </is>
       </c>
       <c r="E1009" t="inlineStr">
@@ -38090,7 +38090,7 @@
       </c>
       <c r="D1016" t="inlineStr">
         <is>
-          <t>존스미스경과 스미스부인</t>
+          <t>존 스미스경과 스미스 부인</t>
         </is>
       </c>
       <c r="E1016" t="inlineStr">
@@ -38128,7 +38128,7 @@
       </c>
       <c r="D1017" t="inlineStr">
         <is>
-          <t>이 예문에서 'advocate'는 '변호사'의 의미로 쓰였습니다. 자연스러운 한국어 문장으로 다듬어 주세요.  [초안]</t>
+          <t>그녀가 그녀의 변호사와 함께 일을 하게 되면서, 그녀는 더욱더 확신을 가지게 되었습니다.</t>
         </is>
       </c>
       <c r="E1017" t="inlineStr">
@@ -38165,6 +38165,27 @@
           <t>Since he put on weight, his jeans have been a tight fit.</t>
         </is>
       </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>그가 몸무게가 늘었기 때문에, 그의 청바지가 더욱 타이트한 핏이 되었습니다.</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>fit = 맞는. 예문 속 문맥과 함께 뜻을 기억하세요.</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr"/>
     </row>
     <row r="1019">
       <c r="A1019" t="inlineStr">
@@ -38182,6 +38203,27 @@
           <t>Show all the spoils by valiant kings achieved.</t>
         </is>
       </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>이 예문에서 'achieve'는 '성취하다'의 의미로 쓰였습니다. 자연스러운 한국어 문장으로 다듬어 주세요.  [초안]</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>achieve = 성취하다. 예문 속 문맥과 함께 뜻을 기억하세요.</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="H1019" t="inlineStr"/>
     </row>
     <row r="1020">
       <c r="A1020" t="inlineStr">
@@ -73929,7 +73971,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D413"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.39999961853027" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.39999961853027"/>
   <cols>
     <col width="16" customWidth="1" style="29" min="1" max="2"/>
     <col width="38.69921875" customWidth="1" style="29" min="3" max="4"/>
@@ -83033,7 +83075,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="29" min="1" max="1"/>
     <col width="70" customWidth="1" style="29" min="2" max="2"/>
@@ -83142,8 +83184,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="29" min="1" max="1"/>
     <col width="24" customWidth="1" style="29" min="2" max="2"/>
@@ -83286,6 +83328,23 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-07 13:14:53</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dictionary_editor_qt_v2.5</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Saved from Editor v2.5 Production Mode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(editor): integrate all dictionary editor productivity features
dictionary_editor_qt.py
Knowledge Engine
Natural Translation Engine
Translation Memory
Phrase Dictionary
Noun Phrases
Verb Patterns
Auto Assist
Golden 저장
Confidence / 추천 이유
</commit_message>
<xml_diff>
--- a/data/words_v3_exampleko_502_1001.xlsx
+++ b/data/words_v3_exampleko_502_1001.xlsx
@@ -37573,7 +37573,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1002" t="inlineStr"/>
     </row>
     <row r="1003">
       <c r="A1003" t="inlineStr">
@@ -37611,7 +37610,6 @@
           <t>Business</t>
         </is>
       </c>
-      <c r="H1003" t="inlineStr"/>
     </row>
     <row r="1004">
       <c r="A1004" t="inlineStr">
@@ -37649,7 +37647,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1004" t="inlineStr"/>
     </row>
     <row r="1005">
       <c r="A1005" t="inlineStr">
@@ -37688,7 +37685,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1005" t="inlineStr"/>
     </row>
     <row r="1006">
       <c r="A1006" t="inlineStr">
@@ -37726,7 +37722,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1006" t="inlineStr"/>
     </row>
     <row r="1007">
       <c r="A1007" t="inlineStr">
@@ -37764,7 +37759,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1007" t="inlineStr"/>
     </row>
     <row r="1008">
       <c r="A1008" t="inlineStr">
@@ -37803,7 +37797,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1008" t="inlineStr"/>
     </row>
     <row r="1009">
       <c r="A1009" t="inlineStr">
@@ -37841,7 +37834,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1009" t="inlineStr"/>
     </row>
     <row r="1010">
       <c r="A1010" t="inlineStr">
@@ -37879,7 +37871,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1010" t="inlineStr"/>
     </row>
     <row r="1011">
       <c r="A1011" t="inlineStr">
@@ -37917,7 +37908,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1011" t="inlineStr"/>
     </row>
     <row r="1012">
       <c r="A1012" t="inlineStr">
@@ -37955,7 +37945,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1012" t="inlineStr"/>
     </row>
     <row r="1013">
       <c r="A1013" t="inlineStr">
@@ -37993,7 +37982,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1013" t="inlineStr"/>
     </row>
     <row r="1014">
       <c r="A1014" t="inlineStr">
@@ -38031,7 +38019,6 @@
           <t>Travel</t>
         </is>
       </c>
-      <c r="H1014" t="inlineStr"/>
     </row>
     <row r="1015">
       <c r="A1015" t="inlineStr">
@@ -38070,7 +38057,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1015" t="inlineStr"/>
     </row>
     <row r="1016">
       <c r="A1016" t="inlineStr">
@@ -38108,7 +38094,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1016" t="inlineStr"/>
     </row>
     <row r="1017">
       <c r="A1017" t="inlineStr">
@@ -38147,7 +38132,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1017" t="inlineStr"/>
     </row>
     <row r="1018">
       <c r="A1018" t="inlineStr">
@@ -38185,7 +38169,6 @@
           <t>Daily</t>
         </is>
       </c>
-      <c r="H1018" t="inlineStr"/>
     </row>
     <row r="1019">
       <c r="A1019" t="inlineStr">
@@ -38205,7 +38188,7 @@
       </c>
       <c r="D1019" t="inlineStr">
         <is>
-          <t>이 예문에서 'achieve'는 '성취하다'의 의미로 쓰였습니다. 자연스러운 한국어 문장으로 다듬어 주세요.  [초안]</t>
+          <t>용맹한 왕들이 이룬 모든 전리품을 보여주세요.</t>
         </is>
       </c>
       <c r="E1019" t="inlineStr">
@@ -38241,6 +38224,27 @@
           <t>Shoulder the blame.</t>
         </is>
       </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>비난을 어깨에 짊어지다(=총대를 메다, 죄를 뒤집어 쓰다)</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>shoulder = 어깨. 예문 속 문맥과 함께 뜻을 기억하세요.</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr"/>
     </row>
     <row r="1021">
       <c r="A1021" t="inlineStr">
@@ -38258,6 +38262,27 @@
           <t>Should we classify "make up" as an idiom or as a phrasal verb?</t>
         </is>
       </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>"make up"을 관용구로 분류해야 할까요, 아니면 구술 동사로 분류해야 할까요?</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>classify = 분류하다. 예문 속 문맥과 함께 뜻을 기억하세요.</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="H1021" t="inlineStr"/>
     </row>
     <row r="1022">
       <c r="A1022" t="inlineStr">
@@ -38275,6 +38300,27 @@
           <t>She's the first athlete in her sport to obtain a corporate sponsor.</t>
         </is>
       </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>athlete가 '운동가'의 뜻으로 쓰인 예문입니다. 문맥에 맞게 한국어로 다듬어 주세요.  [초안]</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>athlete = 운동가. 예문 속 문맥과 함께 뜻을 기억하세요.</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="H1022" t="inlineStr"/>
     </row>
     <row r="1023">
       <c r="A1023" t="inlineStr">
@@ -83184,7 +83230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="29" min="1" max="1"/>
@@ -83345,6 +83391,40 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:16:50</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>dictionary_editor_qt_v2.5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Saved from Editor v2.5 Production Mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-07 15:36:11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>dictionary_editor_qt_v2.5</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Saved from Editor v2.5 Production Mode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>